<commit_message>
Record failed SVPR gate and refresh final assets
</commit_message>
<xml_diff>
--- a/outputs/final_assets/SA-TPA_Final_Experiment_Assets.xlsx
+++ b/outputs/final_assets/SA-TPA_Final_Experiment_Assets.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rf72255b485d5452d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office31 Main" sheetId="2" r:id="Rcbe87ce97d594ee6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OfficeHome Main" sheetId="3" r:id="R578a9b1f5e854b31"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backbone" sheetId="4" r:id="Rca94243a8172434f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ablations" sheetId="5" r:id="Ra75bdba5448943c4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="6" r:id="Ra06054425e2d4879"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Efficiency" sheetId="7" r:id="R4903aff8abf84b1d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bootstrap" sheetId="8" r:id="R352821ab49e94296"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Design Validation" sheetId="9" r:id="R83334f0c709a4739"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Baseline Settings" sheetId="10" r:id="R6a54e436d51d4096"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="11" r:id="R96bcb91488a647d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R839aac2ce2b14c20"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office31 Main" sheetId="2" r:id="R7fc9dc1062684dfb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OfficeHome Main" sheetId="3" r:id="Ree7b7a080e32445a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backbone" sheetId="4" r:id="Rfee0feb132894adf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ablations" sheetId="5" r:id="Rffe6a35c434a4bf6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="6" r:id="Rf7117f23f4294288"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Efficiency" sheetId="7" r:id="R82637f81076c47fb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bootstrap" sheetId="8" r:id="Re5fc8a28c05345fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Design Validation" sheetId="9" r:id="R41a5f2c4e5614d8f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Baseline Settings" sheetId="10" r:id="R975ab886acb54a3d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="11" r:id="Reb58de9981054168"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -238,7 +238,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="90">
+  <x:cellXfs count="84">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -461,24 +461,6 @@
       <x:alignment horizontal="right" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="201" fontId="8" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="201" fontId="8" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="201" fontId="8" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="201" fontId="8" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="201" fontId="8" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="201" fontId="8" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="201" fontId="8" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="right" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -663,7 +645,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R76e72e18c76d4783"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R27510a3a650e4293"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1096,7 +1078,7 @@
     <x:mergeCell ref="G5:H6"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf79dbcd9ea544f5d"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R529b395aa32645ea"/>
 </x:worksheet>
 </file>
 
@@ -1115,16 +1097,16 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
-      <x:c r="A1" s="87" t="str">
+      <x:c r="A1" s="81" t="str">
         <x:v>Baseline Setting Compatibility</x:v>
       </x:c>
-      <x:c r="B1" s="87"/>
-      <x:c r="C1" s="87"/>
-      <x:c r="D1" s="87"/>
-      <x:c r="E1" s="87"/>
-      <x:c r="F1" s="87"/>
-      <x:c r="G1" s="87"/>
-      <x:c r="H1" s="87"/>
+      <x:c r="B1" s="81"/>
+      <x:c r="C1" s="81"/>
+      <x:c r="D1" s="81"/>
+      <x:c r="E1" s="81"/>
+      <x:c r="F1" s="81"/>
+      <x:c r="G1" s="81"/>
+      <x:c r="H1" s="81"/>
     </x:row>
     <x:row r="2" ht="30" customHeight="1">
       <x:c r="A2" s="23" t="str">
@@ -1414,128 +1396,142 @@
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="89" t="str">
+      <x:c r="A4" s="83" t="str">
         <x:v>Office-31 main</x:v>
       </x:c>
-      <x:c r="B4" s="89" t="str">
+      <x:c r="B4" s="83" t="str">
         <x:v>Frozen result</x:v>
       </x:c>
-      <x:c r="C4" s="89" t="str">
+      <x:c r="C4" s="83" t="str">
         <x:v>D:/456/results/office31/development_v2.csv</x:v>
       </x:c>
-      <x:c r="D4" s="89" t="str">
+      <x:c r="D4" s="83" t="str">
         <x:v>ViT-B/32, six tasks</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="89" t="str">
+      <x:c r="A5" s="83" t="str">
         <x:v>Office-Home main</x:v>
       </x:c>
-      <x:c r="B5" s="89" t="str">
+      <x:c r="B5" s="83" t="str">
         <x:v>Frozen result</x:v>
       </x:c>
-      <x:c r="C5" s="89" t="str">
+      <x:c r="C5" s="83" t="str">
         <x:v>D:/456/results/officehome/confirmatory_v1.csv</x:v>
       </x:c>
-      <x:c r="D5" s="89" t="str">
+      <x:c r="D5" s="83" t="str">
         <x:v>ViT-B/32, twelve tasks</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="89" t="str">
+      <x:c r="A6" s="83" t="str">
         <x:v>ViT-B/16</x:v>
       </x:c>
-      <x:c r="B6" s="89" t="str">
+      <x:c r="B6" s="83" t="str">
         <x:v>Kaggle extension</x:v>
       </x:c>
-      <x:c r="C6" s="89" t="str">
+      <x:c r="C6" s="83" t="str">
         <x:v>D:/456/results/vitb16/vitb16_summary.csv</x:v>
       </x:c>
-      <x:c r="D6" s="89" t="str">
+      <x:c r="D6" s="83" t="str">
         <x:v>Completed Kaggle version 5</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="89" t="str">
+      <x:c r="A7" s="83" t="str">
         <x:v>Bootstrap</x:v>
       </x:c>
-      <x:c r="B7" s="89" t="str">
+      <x:c r="B7" s="83" t="str">
         <x:v>Statistical audit</x:v>
       </x:c>
-      <x:c r="C7" s="89" t="str">
+      <x:c r="C7" s="83" t="str">
         <x:v>D:/456/results/robustness/clustered_bootstrap/clustered_bootstrap_summary.csv</x:v>
       </x:c>
-      <x:c r="D7" s="89" t="str">
+      <x:c r="D7" s="83" t="str">
         <x:v>Shared-target corrected</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="89" t="str">
+      <x:c r="A8" s="83" t="str">
         <x:v>Freeze manifest</x:v>
       </x:c>
-      <x:c r="B8" s="89" t="str">
+      <x:c r="B8" s="83" t="str">
         <x:v>Integrity</x:v>
       </x:c>
-      <x:c r="C8" s="89" t="str">
+      <x:c r="C8" s="83" t="str">
         <x:v>D:/456/project/docs/experiment_freeze_manifest.md</x:v>
       </x:c>
-      <x:c r="D8" s="89" t="str">
+      <x:c r="D8" s="83" t="str">
         <x:v>Tag experiments-final-v1</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="89" t="str">
+      <x:c r="A9" s="83" t="str">
         <x:v>Data replica audit</x:v>
       </x:c>
-      <x:c r="B9" s="89" t="str">
+      <x:c r="B9" s="83" t="str">
         <x:v>Data audit</x:v>
       </x:c>
-      <x:c r="C9" s="89" t="str">
+      <x:c r="C9" s="83" t="str">
         <x:v>D:/456/project/docs/data_replica_audit.md</x:v>
       </x:c>
-      <x:c r="D9" s="89" t="str">
+      <x:c r="D9" s="83" t="str">
         <x:v>Raw-image byte identity not asserted</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="89" t="str">
+      <x:c r="A10" s="83" t="str">
         <x:v>Claims evidence index</x:v>
       </x:c>
-      <x:c r="B10" s="89" t="str">
+      <x:c r="B10" s="83" t="str">
         <x:v>Claim traceability</x:v>
       </x:c>
-      <x:c r="C10" s="89" t="str">
+      <x:c r="C10" s="83" t="str">
         <x:v>D:/456/project/docs/claims_evidence_index.md</x:v>
       </x:c>
-      <x:c r="D10" s="89" t="str">
+      <x:c r="D10" s="83" t="str">
         <x:v>Each allowed claim mapped to frozen evidence</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="89" t="str">
+      <x:c r="A11" s="83" t="str">
+        <x:v>SVPR audit</x:v>
+      </x:c>
+      <x:c r="B11" s="83" t="str">
+        <x:v>Post-freeze design validation</x:v>
+      </x:c>
+      <x:c r="C11" s="83" t="str">
+        <x:v>D:/456/project/docs/svpr_experiment_audit.md</x:v>
+      </x:c>
+      <x:c r="D11" s="83" t="str">
+        <x:v>Rejected at corrected three-task development gate</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="83" t="str">
         <x:v>DPA</x:v>
       </x:c>
-      <x:c r="B11" s="89" t="str">
+      <x:c r="B12" s="83" t="str">
         <x:v>Official competitor</x:v>
       </x:c>
-      <x:c r="C11" s="89" t="str">
+      <x:c r="C12" s="83" t="str">
         <x:v>https://openaccess.thecvf.com/content/WACV2025/html/Ali_DPA_Dual_Prototypes_Alignment_for_Unsupervised_Adaptation_of_Vision-Language_Models_WACV_2025_paper.html</x:v>
       </x:c>
-      <x:c r="D11" s="89" t="str">
+      <x:c r="D12" s="83" t="str">
         <x:v>Different source-free, gradient-based setting</x:v>
       </x:c>
     </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="89" t="str">
+    <x:row r="13">
+      <x:c r="A13" s="83" t="str">
         <x:v>DPE</x:v>
       </x:c>
-      <x:c r="B12" s="89" t="str">
+      <x:c r="B13" s="83" t="str">
         <x:v>Official competitor</x:v>
       </x:c>
-      <x:c r="C12" s="89" t="str">
+      <x:c r="C13" s="83" t="str">
         <x:v>https://github.com/zhangce01/DPE-CLIP</x:v>
       </x:c>
-      <x:c r="D12" s="89" t="str">
+      <x:c r="D13" s="83" t="str">
         <x:v>Online TTA; different protocol</x:v>
       </x:c>
     </x:row>
@@ -3453,13 +3449,13 @@
       <x:c r="G5" s="58" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="H5" s="84" t="n">
+      <x:c r="H5" s="58" t="n">
         <x:v>0.7336410080393155</x:v>
       </x:c>
-      <x:c r="I5" s="84" t="n">
+      <x:c r="I5" s="58" t="n">
         <x:v>2.442104911804199</x:v>
       </x:c>
-      <x:c r="J5" s="84" t="n">
+      <x:c r="J5" s="58" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="K5" s="78" t="n">
@@ -3488,13 +3484,13 @@
       <x:c r="G6" s="59" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="H6" s="85" t="n">
+      <x:c r="H6" s="59" t="n">
         <x:v>0.0846463575959205</x:v>
       </x:c>
-      <x:c r="I6" s="85" t="n">
+      <x:c r="I6" s="59" t="n">
         <x:v>1.9497203022241587</x:v>
       </x:c>
-      <x:c r="J6" s="85" t="n">
+      <x:c r="J6" s="59" t="n">
         <x:v>0.0106</x:v>
       </x:c>
       <x:c r="K6" s="79" t="n">
@@ -3523,13 +3519,13 @@
       <x:c r="G7" s="59" t="n">
         <x:v>0.8394</x:v>
       </x:c>
-      <x:c r="H7" s="85" t="n">
+      <x:c r="H7" s="59" t="n">
         <x:v>-3.531235999365648</x:v>
       </x:c>
-      <x:c r="I7" s="85" t="n">
+      <x:c r="I7" s="59" t="n">
         <x:v>1.928750252226988</x:v>
       </x:c>
-      <x:c r="J7" s="85" t="n">
+      <x:c r="J7" s="59" t="n">
         <x:v>0.6312</x:v>
       </x:c>
       <x:c r="K7" s="79" t="n">
@@ -3558,13 +3554,13 @@
       <x:c r="G8" s="59" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="H8" s="85" t="n">
+      <x:c r="H8" s="59" t="n">
         <x:v>0.5086667007766664</x:v>
       </x:c>
-      <x:c r="I8" s="85" t="n">
+      <x:c r="I8" s="59" t="n">
         <x:v>1.124169815704226</x:v>
       </x:c>
-      <x:c r="J8" s="85" t="n">
+      <x:c r="J8" s="59" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="K8" s="79" t="n">
@@ -3593,13 +3589,13 @@
       <x:c r="G9" s="59" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="H9" s="85" t="n">
+      <x:c r="H9" s="59" t="n">
         <x:v>0.1263851393217919</x:v>
       </x:c>
-      <x:c r="I9" s="85" t="n">
+      <x:c r="I9" s="59" t="n">
         <x:v>0.7262328291311859</x:v>
       </x:c>
-      <x:c r="J9" s="85" t="n">
+      <x:c r="J9" s="59" t="n">
         <x:v>0.0032</x:v>
       </x:c>
       <x:c r="K9" s="79" t="n">
@@ -3628,13 +3624,13 @@
       <x:c r="G10" s="60" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="H10" s="86" t="n">
+      <x:c r="H10" s="60" t="n">
         <x:v>3.222786039672792</x:v>
       </x:c>
-      <x:c r="I10" s="86" t="n">
+      <x:c r="I10" s="60" t="n">
         <x:v>9.333150580525398</x:v>
       </x:c>
-      <x:c r="J10" s="86" t="n">
+      <x:c r="J10" s="60" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="K10" s="80" t="n">
@@ -3663,14 +3659,14 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
-      <x:c r="A1" s="87" t="str">
+      <x:c r="A1" s="81" t="str">
         <x:v>Controlled Extension Decisions</x:v>
       </x:c>
-      <x:c r="B1" s="87"/>
-      <x:c r="C1" s="87"/>
-      <x:c r="D1" s="87"/>
-      <x:c r="E1" s="87"/>
-      <x:c r="F1" s="87"/>
+      <x:c r="B1" s="81"/>
+      <x:c r="C1" s="81"/>
+      <x:c r="D1" s="81"/>
+      <x:c r="E1" s="81"/>
+      <x:c r="F1" s="81"/>
     </x:row>
     <x:row r="2" ht="30" customHeight="1">
       <x:c r="A2" s="23" t="str">
@@ -3783,22 +3779,42 @@
       </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="52" t="str">
+      <x:c r="A9" s="49" t="str">
         <x:v>SPT-SA optimal transport</x:v>
       </x:c>
-      <x:c r="B9" s="53" t="str">
+      <x:c r="B9" s="50" t="str">
         <x:v>Office-31, 3 development tasks</x:v>
       </x:c>
-      <x:c r="C9" s="60" t="n">
+      <x:c r="C9" s="59" t="n">
         <x:v>84.06668408115151</x:v>
       </x:c>
-      <x:c r="D9" s="60" t="n">
+      <x:c r="D9" s="59" t="n">
         <x:v>83.905399160086</x:v>
       </x:c>
-      <x:c r="E9" s="60" t="n">
+      <x:c r="E9" s="59" t="n">
         <x:v>-0.1612849210655014</x:v>
       </x:c>
-      <x:c r="F9" s="66" t="str">
+      <x:c r="F9" s="65" t="str">
+        <x:v>Reject at gate</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="52" t="str">
+        <x:v>SVPR prompt weighting (best kappa=20)</x:v>
+      </x:c>
+      <x:c r="B10" s="53" t="str">
+        <x:v>Office-31, 3 development tasks</x:v>
+      </x:c>
+      <x:c r="C10" s="60" t="n">
+        <x:v>84.06668408115151</x:v>
+      </x:c>
+      <x:c r="D10" s="60" t="n">
+        <x:v>84.13870860431835</x:v>
+      </x:c>
+      <x:c r="E10" s="60" t="n">
+        <x:v>0.07202452316684571</x:v>
+      </x:c>
+      <x:c r="F10" s="66" t="str">
         <x:v>Reject at gate</x:v>
       </x:c>
     </x:row>

</xml_diff>